<commit_message>
Import/Export in der App: fachliche Schlüssel, Vorschau-Import, Excel-Export
- Neue App datenaustausch unter /daten/: Vorlage-Download, Gesamtimport
  mit Vorschau (Probelauf mit Rollback, alles-oder-nichts) und
  Gesamtexport als wieder importierbare Mehr-Blatt-Excel-Mappe
- Resources auf Vorlagenformat umgestellt: deutsche Spalten, Klartext-
  Werte (Ja/Nein, Labels, 40 %), fachliche Schlüssel statt DB-PKs
  (Träger-Id, Einrichtungs-Id/Stellen-Id + Name, Personalnummer, E-Mail)
- Sammel-Ids: Einrichtungs-/Stellen-Id dürfen mehrfach vorkommen,
  eindeutig über Id + Name; Vorlage um Namens-Spalten erweitert
- Id-Felder Pflicht + bedingte UniqueConstraints (Migration traeger/0008)
- Excel-Export-Button auf allen Listenseiten (mit Suchfilter)
- Rechte: Import/Export nur Sachbearbeitung/Administration
- 9 Tests (Roundtrip, Idempotenz, Sammel-Id, Transaktionsverhalten)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/import_vorlagen/Stammdaten-Import-Vorlage.xlsx
+++ b/import_vorlagen/Stammdaten-Import-Vorlage.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,6 +87,9 @@
       <b val="1"/>
       <color rgb="001F4E78"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -147,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -182,6 +185,10 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -842,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B21"/>
+  <dimension ref="B1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -965,6 +972,51 @@
       <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Gelb hinterlegte Spalten sind die Schlüssel-Spalten, auf die sich andere Blätter beziehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Sammel-Ids:</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>• Dieselbe Einrichtungs-Id oder Stellen-Id darf für MEHRERE Einrichtungen/Stellen verwendet werden (Sammel-Id, z. B. 16393).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>• Damit der Verweis dann eindeutig ist: im Blatt 'Stellen' zusätzlich die Spalte 'Einrichtung (Name)' ausfüllen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  im Blatt 'Einsätze' die Spalte 'Stelle (Name)'. Bei eindeutigen Ids können diese Spalten leer bleiben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>• Innerhalb einer Sammel-Id muss der Name eindeutig sein – erkannt wird ein Datensatz an Id + Name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>• Die Träger-Id muss weiterhin pro Träger eindeutig sein.</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1508,6 +1560,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1561,6 +1614,11 @@
           <t>optional</t>
         </is>
       </c>
+      <c r="K1" s="13" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
@@ -1613,6 +1671,11 @@
           <t>Bemerkung</t>
         </is>
       </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>Einrichtung (Name)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -1657,6 +1720,11 @@
         </is>
       </c>
       <c r="J3" s="9" t="inlineStr"/>
+      <c r="K3" s="15" t="inlineStr">
+        <is>
+          <t>Kita Sonnenschein</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2056,7 +2124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2067,6 +2135,7 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2110,6 +2179,11 @@
           <t>optional</t>
         </is>
       </c>
+      <c r="I1" s="13" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
@@ -2152,6 +2226,11 @@
           <t>Bemerkung</t>
         </is>
       </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>Stelle (Name)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -2186,6 +2265,11 @@
         </is>
       </c>
       <c r="H3" s="9" t="inlineStr"/>
+      <c r="I3" s="15" t="inlineStr">
+        <is>
+          <t>Gemeindediakon</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
Excel-Exporte und Import-Vorlage in ELKB-CI-Farben
Kopfzeile Violett #5B2281, Markerzeile Blaugrau #839ABA, Schlüsselspalten
Hellviolett #C8B8DB, dezente Zeilenstreifen #ECE7F3 – wie das App-Theme.
Anleitungstext der Vorlage angepasst (Schlüsselspalten violett statt gelb).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/import_vorlagen/Stammdaten-Import-Vorlage.xlsx
+++ b/import_vorlagen/Stammdaten-Import-Vorlage.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,8 +90,21 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="005B2281"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="005B2281"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +136,21 @@
         <fgColor rgb="00A6A6A6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00839ABA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B2281"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8B8DB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -150,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -189,6 +217,20 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -849,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B28"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -857,12 +899,13 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Stammdaten-Import – Vorlage für das Diakon-CRM</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -912,6 +955,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -926,6 +970,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -968,16 +1013,15 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Gelb hinterlegte Spalten sind die Schlüssel-Spalten, auf die sich andere Blätter beziehen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" t="inlineStr"/>
-    </row>
+          <t>Hell-violett hinterlegte Spalten sind die Schlüssel-Spalten, auf die sich andere Blätter beziehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
     <row r="23">
       <c r="B23" s="12" t="inlineStr">
         <is>
@@ -1044,74 +1088,74 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="D1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="E1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Vorname</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Nachname</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
         <is>
           <t>Geschlecht</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>E-Mail</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>Telefon</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="18" t="inlineStr">
         <is>
           <t>Notiz</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="18" t="inlineStr">
         <is>
           <t>Aktiv</t>
         </is>
@@ -1189,94 +1233,94 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="D1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="E1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="H1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="I1" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Träger-Id</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
         <is>
           <t>Art</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>Haupt-Ansprechpartner (E-Mail)</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>Straße</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="18" t="inlineStr">
         <is>
           <t>PLZ</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="18" t="inlineStr">
         <is>
           <t>Ort</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="18" t="inlineStr">
         <is>
           <t>Aktiv</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="18" t="inlineStr">
         <is>
           <t>Bemerkung</t>
         </is>
@@ -1362,114 +1406,114 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="E1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="H1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="I1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="J1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="I1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="J1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="K1" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Einrichtungs-Id</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
         <is>
           <t>Träger-Id</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>Art</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>Straße</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="18" t="inlineStr">
         <is>
           <t>PLZ</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="18" t="inlineStr">
         <is>
           <t>Ort</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="18" t="inlineStr">
         <is>
           <t>Ansprechpartner (E-Mail)</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="18" t="inlineStr">
         <is>
           <t>Versorgungsumlage</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="18" t="inlineStr">
         <is>
           <t>Aktiv</t>
         </is>
       </c>
-      <c r="K2" s="8" t="inlineStr">
+      <c r="K2" s="18" t="inlineStr">
         <is>
           <t>Bemerkung</t>
         </is>
@@ -1564,114 +1608,114 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="E1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="H1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="I1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="J1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="K1" s="13" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="I1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="J1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="K1" s="20" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Stellen-Id</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
         <is>
           <t>Einrichtungs-Id</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>Straße</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="18" t="inlineStr">
         <is>
           <t>PLZ</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="18" t="inlineStr">
         <is>
           <t>Ort</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="18" t="inlineStr">
         <is>
           <t>Ansprechpartner (E-Mail)</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="18" t="inlineStr">
         <is>
           <t>Aktiv</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="18" t="inlineStr">
         <is>
           <t>Bemerkung</t>
         </is>
       </c>
-      <c r="K2" s="14" t="inlineStr">
+      <c r="K2" s="21" t="inlineStr">
         <is>
           <t>Einrichtung (Name)</t>
         </is>
@@ -1770,214 +1814,214 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="H1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="I1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="J1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="K1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="L1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="M1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="N1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="O1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="P1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="Q1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="R1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="S1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="T1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="U1" s="7" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="I1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="J1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="K1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="L1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="M1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="N1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="O1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="P1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="Q1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="R1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="S1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="T1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="U1" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Personalnummer</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Geschlecht</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
         <is>
           <t>Vorname</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>Nachname</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>Geburtsdatum</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="18" t="inlineStr">
         <is>
           <t>E-Mail</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="18" t="inlineStr">
         <is>
           <t>Telefon privat</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="18" t="inlineStr">
         <is>
           <t>Telefon dienstlich</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="18" t="inlineStr">
         <is>
           <t>Straße</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="18" t="inlineStr">
         <is>
           <t>PLZ</t>
         </is>
       </c>
-      <c r="K2" s="8" t="inlineStr">
+      <c r="K2" s="18" t="inlineStr">
         <is>
           <t>Ort</t>
         </is>
       </c>
-      <c r="L2" s="8" t="inlineStr">
+      <c r="L2" s="18" t="inlineStr">
         <is>
           <t>Anstellung</t>
         </is>
       </c>
-      <c r="M2" s="8" t="inlineStr">
+      <c r="M2" s="18" t="inlineStr">
         <is>
           <t>Dienststand</t>
         </is>
       </c>
-      <c r="N2" s="8" t="inlineStr">
+      <c r="N2" s="18" t="inlineStr">
         <is>
           <t>Besoldungsgruppe</t>
         </is>
       </c>
-      <c r="O2" s="8" t="inlineStr">
+      <c r="O2" s="18" t="inlineStr">
         <is>
           <t>Stufe</t>
         </is>
       </c>
-      <c r="P2" s="8" t="inlineStr">
+      <c r="P2" s="18" t="inlineStr">
         <is>
           <t>Familienstand</t>
         </is>
       </c>
-      <c r="Q2" s="8" t="inlineStr">
+      <c r="Q2" s="18" t="inlineStr">
         <is>
           <t>Kinder</t>
         </is>
       </c>
-      <c r="R2" s="8" t="inlineStr">
+      <c r="R2" s="18" t="inlineStr">
         <is>
           <t>Kindergeldberechtigt</t>
         </is>
       </c>
-      <c r="S2" s="8" t="inlineStr">
+      <c r="S2" s="18" t="inlineStr">
         <is>
           <t>Voller OFZ-Anspruch</t>
         </is>
       </c>
-      <c r="T2" s="8" t="inlineStr">
+      <c r="T2" s="18" t="inlineStr">
         <is>
           <t>Aktiv</t>
         </is>
       </c>
-      <c r="U2" s="8" t="inlineStr">
+      <c r="U2" s="18" t="inlineStr">
         <is>
           <t>Bemerkung</t>
         </is>
@@ -2139,94 +2183,94 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>PFLICHT</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="E1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="H1" s="7" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="I1" s="13" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Stellen-Id</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="19" t="inlineStr">
         <is>
           <t>Personalnummer</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
         <is>
           <t>Beginn</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>Ende</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>Umfang</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="18" t="inlineStr">
         <is>
           <t>Abrechnung über LKA</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="18" t="inlineStr">
         <is>
           <t>Aktiv</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="18" t="inlineStr">
         <is>
           <t>Bemerkung</t>
         </is>
       </c>
-      <c r="I2" s="14" t="inlineStr">
+      <c r="I2" s="21" t="inlineStr">
         <is>
           <t>Stelle (Name)</t>
         </is>

</xml_diff>

<commit_message>
mbw: Storno-Matching verbessern, Rechnungstext-Kopf, Stammdaten-Export
Storno-Matching (sap_import): +/- Paarung reihenfolge-unabhängig (SAP bucht
Storno oft vor Neubuchung) und RV-Gegenbuchungen über zwei Lohnarten
(1S32/9V98, /361/9V61, /363/9V63) zusammenklappen. Angezeigte Summen zählen
nur noch sichtbare Zeilen; Kontosummen bleiben unverändert. Wirkt erst nach
erneutem SAP-Import.

Rechnungstexte (Abschlag + Spitze): neuer Kopf im gewünschten Format
(Pers.Nr., Titel/Name, Einsatz mit Träger und Einsatzort, Umfang, Stellen-ID,
von/bis, Art der Rechnung, Standard-Anrede).

Datenaustausch: Debitoren und Innenaufträge roundtrip-fähig im
Gesamtexport/-import (mbw/resources.py, registry, Import-Vorlage). Debitor
über interne Id, Innenauftrag über Nummer; Einsatz-Bezug read-only.

Tests: 42 grün (mbw 30 + datenaustausch 12).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/import_vorlagen/Stammdaten-Import-Vorlage.xlsx
+++ b/import_vorlagen/Stammdaten-Import-Vorlage.xlsx
@@ -14,6 +14,8 @@
     <sheet name="Stellen" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Mitarbeiter" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Einsätze" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Debitoren" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Innenaufträge" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -178,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -231,6 +233,7 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -891,7 +894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="B1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -905,7 +908,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -955,7 +957,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -970,7 +971,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -1013,7 +1013,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
@@ -1021,7 +1020,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="B23" s="12" t="inlineStr">
         <is>
@@ -2327,4 +2325,364 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>PFLICHT</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="J1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="K1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="L1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="M1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>SAP-Debitorennummer</t>
+        </is>
+      </c>
+      <c r="C2" s="22" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>Namenszusatz</t>
+        </is>
+      </c>
+      <c r="E2" s="21" t="inlineStr">
+        <is>
+          <t>Anschriftperson</t>
+        </is>
+      </c>
+      <c r="F2" s="21" t="inlineStr">
+        <is>
+          <t>Straße</t>
+        </is>
+      </c>
+      <c r="G2" s="21" t="inlineStr">
+        <is>
+          <t>PLZ</t>
+        </is>
+      </c>
+      <c r="H2" s="21" t="inlineStr">
+        <is>
+          <t>Ort</t>
+        </is>
+      </c>
+      <c r="I2" s="21" t="inlineStr">
+        <is>
+          <t>E-Mail</t>
+        </is>
+      </c>
+      <c r="J2" s="21" t="inlineStr">
+        <is>
+          <t>Versandweg</t>
+        </is>
+      </c>
+      <c r="K2" s="21" t="inlineStr">
+        <is>
+          <t>Träger-Id</t>
+        </is>
+      </c>
+      <c r="L2" s="21" t="inlineStr">
+        <is>
+          <t>Aktiv</t>
+        </is>
+      </c>
+      <c r="M2" s="21" t="inlineStr">
+        <is>
+          <t>Bemerkung</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1900012345</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Beispiel-Rechnungsanschrift</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>z. Hd. Frau Muster</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Kirchweg 5</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>90000</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Musterstadt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>E-Mail</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>TR-001</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>PFLICHT</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>Innenauftrag</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Bezeichnung</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="inlineStr">
+        <is>
+          <t>Kostenstelle</t>
+        </is>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>Debitor-Id</t>
+        </is>
+      </c>
+      <c r="E2" s="21" t="inlineStr">
+        <is>
+          <t>Aktiv</t>
+        </is>
+      </c>
+      <c r="F2" s="21" t="inlineStr">
+        <is>
+          <t>Bemerkung</t>
+        </is>
+      </c>
+      <c r="G2" s="21" t="inlineStr">
+        <is>
+          <t>Andock-Art</t>
+        </is>
+      </c>
+      <c r="H2" s="21" t="inlineStr">
+        <is>
+          <t>Einsatz (Personalnr.)</t>
+        </is>
+      </c>
+      <c r="I2" s="21" t="inlineStr">
+        <is>
+          <t>Einsatz (Stellen-Id)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F031233-0034</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>3-0312-033</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>an Stelle</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>